<commit_message>
Add round-2 Southwire-published case studies and reorder workbook by relevance
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6BTX8phSjo7v37zFMgeMW
</commit_message>
<xml_diff>
--- a/Southwire_Case_Studies.xlsx
+++ b/Southwire_Case_Studies.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Case Studies'!$A$3:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Case Studies'!$A$3:$I$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,7 +67,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,12 +81,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00F2F7F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F7F2"/>
+        <fgColor rgb="00EEF4FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -96,7 +96,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F5F2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FBEDE6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -126,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -168,6 +178,24 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -544,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -625,42 +653,42 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Southwire as customer</t>
+          <t>Southwire-published (utility)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>SAP Cloud Migration to Google Cloud</t>
+          <t>C7 Overhead Conductor - River Crossing</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Google Cloud / Avvale / NIMBL</t>
+          <t>Southwire</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/customers/southwire</t>
+          <t>https://www.southwire.com/Utility-Whitepapers-CaseStudy</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Upgraded SAP ECC to EhP8, deployed SAP BW on HANA, upgraded SAP Process Orchestration, and migrated the SAP estate to Google Cloud with Avvale and NIMBL under the Google Cloud Acceleration Program.</t>
+          <t>Riverbank erosion forced a support structure move, increasing a river-crossing span from 1,290 ft to 1,840 ft; ACSR would have sagged too much, requiring larger structures and foundations, so the utility used C7 carbon-fiber composite-core conductor.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Only ~22 hours total downtime across 3 SAP systems during a July 4th weekend cutover; system changes that previously needed 1+ hour of SAP downtime now cause zero interruption; keeps 30+ factories running 24/7.</t>
+          <t>Span increased ~43% (1,290 to 1,840 ft) with no increase in sag; avoided full line rebuild and new foundations; 40+ year service-life expectancy; single-failure-tolerant multi-stranded core.</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Near-zero platform downtime, five layers of data protection, performance boost, and a foundation for connected-factory and AI/ML initiatives.</t>
+          <t>Higher capacity and superior sag/tension performance let utilities reuse existing structures and cut total project cost.</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Also see Avvale case study and Google Cloud blog 'Why Southwire migrated'.</t>
+          <t>See also Utility Dive sponsored article on composite core conductors. Directly supports Case 3 (Crossing) in the Advanced Conductor Value Prop deck.</t>
         </is>
       </c>
     </row>
@@ -670,42 +698,42 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Southwire as customer</t>
+          <t>Southwire-published (utility)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Customer Hub Self-Service Portal (SAP Commerce Cloud)</t>
+          <t>Novinium Cable Rejuvenation - Salt River Project</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Southwire (Novinium Underground Services)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>https://www.sap.com/asset/dynamic/2025/05/405f8320-067f-0010-bca6-c68f7e60039b.html</t>
+          <t>https://www.southwire.com/Utility-Whitepapers-CaseStudy</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Digital-first transformation: self-service Customer Hub built on SAP Commerce Cloud, integrated with SAP ERP and SAP BTP; real-time order tracking, product info with variant configuration and pricing.</t>
+          <t>Salt River Project (utility serving south Phoenix, AZ) had aging feeder and URD cable with rising maintenance costs; chose Novinium cable rejuvenation instead of replacement.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Freed customer-service teams from hundreds of thousands of internet queries; customers access real-time information 24/7; new features added with quick turnarounds.</t>
+          <t>Less than 1% post-rejuvenation failure rate.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Removes service bottlenecks - customers self-serve anytime while service staff focus on higher-value work.</t>
+          <t>Rejuvenation extends cable life at a fraction of replacement cost with minimal customer disruption.</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>See also ASUG interview on Southwire's digitalization journey.</t>
+          <t>Salt River Project Whitepaper PDF on southwire.com.</t>
         </is>
       </c>
     </row>
@@ -715,40 +743,44 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Southwire as customer</t>
+          <t>Southwire-published (utility)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Connected Enterprise Digital Transformation ('Southwire Makes the Right Connections')</t>
+          <t>Novinium Modular Injection Component (MIC) - National Grid</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Rockwell Automation</t>
+          <t>Southwire (Novinium Underground Services)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>https://www.rockwellautomation.com/en-us/company/news/case-studies/southwire-digital-transformation.html</t>
+          <t>https://www.southwire.com/Utility-Whitepapers-CaseStudy</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Multi-year Connected Enterprise / IT-OT convergence initiative connecting all insulated and bare wire-and-cable manufacturing, starting with a proof of concept and two-plant pilot.</t>
+          <t>National Grid (Northeast US IOU, 10M+ gas &amp; electric customers in NY/MA/RI, thousands of miles of aging unjacketed XLPE URD cable; SPR injections since 2007) used the MIC - first 200A accessory enabling energized SPR injection of MV cables; developed with Richards Manufacturing.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>~3-year rollout to connect all manufacturing facilities; operators verify device-level quality settings on every run (published outcomes mostly qualitative).</t>
+          <t>5,000+ feet of energized cable segments injected via MIC with sustained-pressure-rejuvenation reliability; full rejuvenation of radial segments within the standard 2-hour outage window normally reserved just for testing; improved crew productivity (crews move on while injection continues).</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Data-driven decisions instead of opinion-driven; measure and manage productivity in new ways; integrated automation enables further innovation.</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr"/>
+          <t>Energized injection means shorter outages, higher crew productivity, less rate-payer disruption than replacement or de-energized rejuvenation.</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Mountain View Electric Association (CO co-op, 50,000+ members, ~600 mi aging URD cable) is a related Novinium injection reference.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="110" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -756,40 +788,44 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Southwire as customer</t>
+          <t>Southwire-published (utility)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>People Analytics for HR ('Igniting HR Operations at Southwire')</t>
+          <t>C7 First Commercial Installation - CenterPoint Energy 138-kV Reconductor</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Crunchr</t>
+          <t>Southwire / T&amp;D World ('High Capacity Meets Low Sag')</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>https://www.crunchr.com/customers/southwire/</t>
+          <t>https://www.tdworld.com/overhead-transmission/article/20964350/high-capacity-meets-low-sag</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>HR team faced scattered, unreliable workforce data; adopted Crunchr people-analytics platform to centralize workforce insights.</t>
+          <t>CenterPoint Energy became the first commercial installer of C7 (carbon-fiber core with Celanese Celstran CFR-TPR) on a 138-kV line between Crosby and Mont Belvieu northeast of Houston - a fast-growing natural-gas-storage area that added six new 138-kV substations in one year. Existing line: single-circuit twin bundle 927.2 kcmil ACAR on double-circuit vertical steel towers.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Platform integrated within ~1 month - significantly faster than the internal-build timeline quoted by Southwire's own BI team.</t>
+          <t>C7 delivers nearly 2x the ampacity of same-diameter ACSR with less sag; reconductor doubled capacity without exceeding existing design tensions or replacing structures.</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Faster, more consistent workforce insights; better decision-making; strong vendor support vs slower internal build.</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr"/>
+          <t>Uprate more lines on existing structures - proof point for the reconductor-vs-rebuild value proposition.</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Directly supports Case 1 (Reconductor vs Rebuild) in the Advanced Conductor Value Prop deck.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="110" customHeight="1">
       <c r="A8" s="4" t="n">
@@ -797,40 +833,44 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Southwire as customer</t>
+          <t>Southwire-published (utility)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>B2B Demand Generation ('Establishing a Digital Baseline')</t>
+          <t>VR2 Vibration-Resistant Conductor - Midwest Utility (Ice Galloping)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Marsden Marketing</t>
+          <t>Southwire Overhead Transmission</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>https://www.marsdenmarketing.com/case-study-establishing-a-digital-baseline</t>
+          <t>https://overheadtransmission.southwire.com/projects/midwest-utility/</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Digital marketing program (microsites, SEO, lead gen) for Southwire's Power Systems &amp; Solutions group across three business verticals.</t>
+          <t>Large Midwest utility in an area with severe aeolian vibration, ice storms, and ice galloping installed VR2 twisted-pair conductor on a 0.65-mile stretch of 69-kV horizontal-post line in 2008 as a side-by-side comparison with traditional twisted-pair construction.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>259% increase in lead database across all three verticals; all three microsites on page 1 of Google for competitive keywords; lead-gen goals exceeded in each vertical.</t>
+          <t>Utility estimated ~$70M restoration cost from the Feb 2007 ice storm; ice can add 6-7x conductor weight; VR2's variable lay length installs without bagging issues while giving equal or better resistance to aeolian vibration and ice galloping.</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Measurable digital baseline and pipeline growth for an industrial B2B business unit.</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr"/>
+          <t>Avoid multimillion-dollar storm-restoration costs by hardening lines against ice galloping - reliability as avoided cost.</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Case study PDF: SW_VR2_Midwest_Utility_Case_Study on overheadtransmission.southwire.com.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="110" customHeight="1">
       <c r="A9" s="4" t="n">
@@ -838,40 +878,44 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Southwire as customer</t>
+          <t>Southwire-published (utility)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Facility Services</t>
+          <t>SIMpull Cable-in-Conduit - Columbia Basin Electric Cooperative</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Millennium Facility Services (MFS / MillenniumOS)</t>
+          <t>Southwire</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>https://millfac.com/case-studies/southwire</t>
+          <t>https://www.southwire.com/newsroom/archive/case-study-going-underground-helps-columbia-basin-electric-cooperative-beat-extreme-weather-ice-storms</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Outsourced facility services across Southwire buildings with autonomous equipment optimization and production-aligned cleaning schedules.</t>
+          <t>Pacific-Northwest co-op facing extreme weather (90 ft mountain snow, 30 in valley rain, 100-degree high desert; fog and ice knocking out overhead service to rural customers for weeks) went underground with SIMpull Cable-in-Conduit: 1/0 stranded 15-kV 220-mil EPR in 1.5-inch Schedule 40 HDPE on 2,500-ft reels.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>11% under contracted budget; 35% reduction in cleaning-related production downtime; 99.7% GPS-verified task-completion rate; 100% Avetta compliance with zero audit deficiencies.</t>
+          <t>60%+ of co-op members now prefer CIC over separate cable-and-conduit installs; faster installs (no PVC joint inspections), no mud/water-clogged conduit issues, reduced labor cost; spare conduit capacity allows pulling a replacement conductor after a failure.</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Lower facility cost with verifiable execution and less interference with production.</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr"/>
+          <t>One-step undergrounding that hardens rural feeders against weather while cutting install labor.</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Re3 SIMpull CIC case study also on CableTechSupport page; CIC used across DOT, DOE, EV infrastructure, grid hardening, airports, renewables, data centers.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="110" customHeight="1">
       <c r="A10" s="4" t="n">
@@ -879,37 +923,37 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Southwire as customer</t>
+          <t>Southwire-published (utility)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Recruitment Marketing - Bremen, IN Plant</t>
+          <t>Vineyard Wind 1 - Onshore HV Cable Supply &amp; Installation</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Federated Media</t>
+          <t>Southwire / Vineyard Wind</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>https://info.federatedmedia.com/southwire-case-study</t>
+          <t>https://www.southwire.com/blogs/vineyard-wind</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>New 250,000 sq ft facility in Bremen, Indiana needed 100 positions filled immediately in a tight labor market; high-frequency radio ads (WRBR, WBYT, WAOR) plus on-site hiring event.</t>
+          <t>Key supplier for design, manufacture, and installation of onshore high-voltage cables for Vineyard Wind 1 - the first commercial-scale US offshore wind farm (800 MW, 84 x 9.5 MW turbines, 15 miles off Martha's Vineyard, powering 400,000+ homes/businesses). Cable made at the 250,000 sq ft Huntersville, NC HV/EHV plant (69-500 kV); installed by Southwire's HV field services team with local labor.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Hiring-event turnout exceeded expectations; job offers extended to 2x as many prospective employees as initially hoped.</t>
+          <t>32+ miles of high-voltage cable manufactured; onshore scope completed ~Q1 2023.</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Fast, high-volume hourly recruitment for a new plant using targeted local media.</t>
+          <t>US-made HV cable plus turnkey field installation for flagship energy-transition projects.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
@@ -920,37 +964,37 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Southwire as customer</t>
+          <t>Southwire-published (utility)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Employee Well-Being (GRI Sustainability Case)</t>
+          <t>Novinium Underground Services - Dayton</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>SustainCase</t>
+          <t>Southwire (Novinium Underground Services)</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>https://sustaincase.com/case-study-how-southwire-promotes-employee-well-being/</t>
+          <t>https://www.southwire.com/Utility-Whitepapers-CaseStudy</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Analysis of how Southwire promotes employee well-being (health, safety, wellness) based on GRI-standard sustainability reporting.</t>
+          <t>Additional Novinium underground cable-rejuvenation deployment (Dayton); companion to the SRP and MIC studies.</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Qualitative; references Southwire's published sustainability metrics (southwire.com Metrics at a Glance).</t>
+          <t>See PDF.</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Employer-of-choice positioning and workforce sustainability as a business asset.</t>
+          <t>Rejuvenate-vs-replace economics applied at another utility.</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
@@ -961,514 +1005,813 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
+          <t>Southwire-published (utility)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Digital Grid Resiliency - Northeast US Investor-Owned Utility</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Southwire</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.southwire.com/services/digital-grid-resiliency-assessments</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Northeast US IOU worked with Southwire over several years, evaluating circuits and applying an enhanced grid-resiliency program to a subset; AI-assisted assessment mines outage and GIS data to classify outage root causes at device level.</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Assessment identifies reliability improvements in as little as 30 days; prescriptive recommendations include cost justification and expected reliability gains.</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Data/AI-driven, device-level targeting of grid-hardening spend instead of blanket programs.</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>'Volatile to Resilient' case study PDF on the whitepapers index; Utility Dive sponsored article.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="110" customHeight="1">
+      <c r="A13" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Southwire-published (services)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>SPEED / CableTechSupport Services - Metals &amp; Mining Corporation (Canada)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Southwire (via Electrical Industry News Week, Nov 2022)</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>https://electricalindustry.ca/latest-articles/8917-case-study-southwire-customizable-speed-and-cabletech-support-services/</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>One of the world's largest metals &amp; mining corporations needed a medium-voltage cable solution in Canada; Southwire delivered a customized, expedited solution combining SPEED services (striping, marking, kitting, labeling, bundling) and the CableTechSupport engineering team.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Published metrics limited in search results; SPEED page lists Expedited Service, Unrivaled Service, and Standard-to-Innovative case studies.</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Engineering support plus expedited, customized cable supply keeps mission-critical industrial projects on schedule.</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>More SPEED case studies at southwire.com/services/speed-services and /services/stock-services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="110" customHeight="1">
+      <c r="A14" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Contractor Solutions / jobsite</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>SIMpull Solutions / Contractor Solutions Program</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Southwire</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>https://www.southwire.com/services/contractor-solutions</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Jobsite productivity system - SIMpull CoilPAK payoffs, SIMpull BARREL drums, SIMpull REEL, NoLube SIMpull THHN, MAXIS pulling equipment - plus Contractor Solutions Professionals (CSPs) consulting on layouts, pulling calcs, and setup for the project duration.</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Up to 50% jobsite efficiency/savings claimed; SIMpull REEL setup ~4x faster (no jack stands, fewer people, multiple runs per reel); MAXIS: 1-man 39-min pull vs 45 min for traditional 2-man setup.</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>Beat branch-circuit wiring budgets by cutting material handling, setup time, and crew size.</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Detailed per-project case studies appear to live with CSP team / Solutions Partner Distributors, not published openly - request internally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="110" customHeight="1">
+      <c r="A15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Contractor Solutions / jobsite</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Data Center Solutions (QWIK Whips, Cabling Solutions)</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Southwire</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>https://www.southwire.com/industries/data-centers</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Pre-assembled QWIK Whip cables and cable-pulling solutions for data center builds; positions Southwire on labor reduction and schedule for hyperscale/AI construction.</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>Publicly qualitative (streamlined ordering/install/assembly, labor cost management); no published quantified project case study found.</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Reduce constrained field labor and keep data center projects on schedule.</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Gap the internal Advanced Conductor Value Prop deck is designed to fill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="110" customHeight="1">
+      <c r="A16" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Contractor Solutions / jobsite</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Contractor Solutions Case Study Library (incl. Aldi Distribution Center)</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Southwire</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>https://www.southwire.com/services/contractor-solutions</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Southwire publishes a series of named jobsite case-study PDFs on the Contractor Solutions page: Aldi Distribution Center; 'Ineffective to Productive' (CSPs proposed an alternative install method using HDPE Schedule 40 conduit with SIMpull Solutions); 'Obstacle to Advantage'; 'Cumbersome to Effective'; 'Standard to Innovative'; 'Time-Consuming to Efficient'; 'Delayed to On Schedule'; 'Harder to Smarter'; 'Complicated to SIMpull'.</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Per-project labor/time savings are inside each PDF (e.g. Aldi-Distribution-Center-Case-Study and Ineffective-Productive-Case-Study on southwire.com/medias); not indexed by search engines.</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Real projects showing SIMpull Solutions + CSP consultation converting jobsite problems into schedule and labor wins - the closest public analog to the quantified-outcome format the Value Prop deck targets.</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Download the PDFs from the Contractor Solutions page for the numbers; also IEEE 'Innovative' case study at southwire.com/ieee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="110" customHeight="1">
+      <c r="A17" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Southwire-published (corporate)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>12 for Life - Harvard Business School Case ('Southwire and 12 For Life: Scaling Up?')</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>Harvard Business School / Southwire</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>https://www.hbs.edu/faculty/Pages/item.aspx?num=45785</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Southwire partnered with the local Georgia school system to staff a factory with at-risk high-school students who combine classroom instruction with paid work in a modified manufacturing environment.</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>Factory runs at a profit while producing remarkable student-outcome improvements; the oldest case of its kind still taught at Harvard Business School.</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>Shared-value proof point: workforce development and community impact that also makes commercial sense.</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>Useful for corporate-credibility slides rather than product ROI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="110" customHeight="1">
+      <c r="A18" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Internal - Adv. Conductor Value Prop</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>C7 Corridor Upgrade - Reconductor vs Rebuild (Illustrative 25-mile Corridor)</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Internal deck (user-shared slides, 2026-08-18)</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr"/>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Executive value-prop model: reconductoring an existing 25-mile corridor with C7 vs traditional new-build. Existing towers and ROW reused - only the conductor changes ('same towers, same right-of-way - a stronger line, delivered in a fraction of the time').</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>~$57.5M capital avoided ($87.5M new-build to $30.0M C7); 6 years faster to capacity (~2 vs ~8 yrs); +450 MVA (2.5x throughput, 300 to 750 MVA). Breakdown: ~$30.0M structures/foundations, ~$15.0M ROW/permitting/legal, ~$7.5M materials efficiency, ~$5.0M labor/construction.</t>
+        </is>
+      </c>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>Faster, lower-risk capacity expansion on corridors the utility already owns - a capacity solution, not a conductor purchase.</t>
+        </is>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>Assumptions: baseline 300 MVA; C7 at 2.5x; structure &amp; ROW reuse; illustrative figures only. Deck defines 4 validation cases: 1) Reconductor vs Rebuild, 2) New Build, 3) Crossing, 4) Line Loss Reduction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="110" customHeight="1">
+      <c r="A19" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Internal - Adv. Conductor Value Prop</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>Prefab Cable for Modular Cooling OEMs (Vertiv-style Archetype)</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Internal deck (user-shared slides, 2026-08-18)</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr"/>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Cooling is the critical path in AI &amp; hyperscale deployments; Southwire prefab electrical scope (skid-mounted, factory-tested, pre-routed power &amp; controls cable, plug-and-play CDU/chiller hookup) vs traditional field integration (field piping/brazing/welding, field-run controls, refrigerant/balancing/testing, multi-trade risk).</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>Onsite deployment 6-10 weeks vs 4-6+ months traditional; 2-4 months schedule compression.</t>
+        </is>
+      </c>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>Earlier customer energization, lower commissioning risk, repeatable across fleets; combined story: accelerate capacity while reducing dependence on constrained field labor.</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>Illustrative; Vertiv referenced as representative modular cooling OEM partner archetype.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="110" customHeight="1">
+      <c r="A20" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Internal - Adv. Conductor Value Prop</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Prefab Cable for Power Distribution Skid Providers</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Internal deck (user-shared slides, 2026-08-18)</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr"/>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Illustrative 50 MW distribution skid deployment block; loaded field labor at $180/hr. Traditional field build (15 electricians x 10 wks; weather/rework/multi-trade risk) vs Southwire prefab (pre-tested, pre-labeled harnesses; plug-and-play modular connections).</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>Install + commissioning 2-4 wks vs 8-12 wks; 40-60% fewer onsite labor hours; per block: 6-8 wks faster to energization, $500K-$800K field labor savings (vs ~$1.1M-$1.5M traditional); lower rework, faster revenue recognition, reduced LD exposure.</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>Faster energization and lower labor cost per repeatable deployment block. Targets: data centers, utility substations, battery storage, AI infrastructure, modular industrial plants, fuel cell &amp; gen-set OEMs.</t>
+        </is>
+      </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>Figures directional - validate with partner labor data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="110" customHeight="1">
+      <c r="A21" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
           <t>Southwire as customer</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>SAP Cloud Migration to Google Cloud</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Google Cloud / Avvale / NIMBL</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/customers/southwire</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>Upgraded SAP ECC to EhP8, deployed SAP BW on HANA, upgraded SAP Process Orchestration, and migrated the SAP estate to Google Cloud with Avvale and NIMBL under the Google Cloud Acceleration Program.</t>
+        </is>
+      </c>
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>Only ~22 hours total downtime across 3 SAP systems during a July 4th weekend cutover; system changes that previously needed 1+ hour of SAP downtime now cause zero interruption; keeps 30+ factories running 24/7.</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>Near-zero platform downtime, five layers of data protection, performance boost, and a foundation for connected-factory and AI/ML initiatives.</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>Also see Avvale case study and Google Cloud blog 'Why Southwire migrated'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="110" customHeight="1">
+      <c r="A22" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Southwire as customer</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>Customer Hub Self-Service Portal (SAP Commerce Cloud)</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>https://www.sap.com/asset/dynamic/2025/05/405f8320-067f-0010-bca6-c68f7e60039b.html</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>Digital-first transformation: self-service Customer Hub built on SAP Commerce Cloud, integrated with SAP ERP and SAP BTP; real-time order tracking, product info with variant configuration and pricing.</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>Freed customer-service teams from hundreds of thousands of internet queries; customers access real-time information 24/7; new features added with quick turnarounds.</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>Removes service bottlenecks - customers self-serve anytime while service staff focus on higher-value work.</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>See also ASUG interview on Southwire's digitalization journey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="110" customHeight="1">
+      <c r="A23" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Southwire as customer</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>Connected Enterprise Digital Transformation ('Southwire Makes the Right Connections')</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Rockwell Automation</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>https://www.rockwellautomation.com/en-us/company/news/case-studies/southwire-digital-transformation.html</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>Multi-year Connected Enterprise / IT-OT convergence initiative connecting all insulated and bare wire-and-cable manufacturing, starting with a proof of concept and two-plant pilot.</t>
+        </is>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>~3-year rollout to connect all manufacturing facilities; operators verify device-level quality settings on every run (published outcomes mostly qualitative).</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>Data-driven decisions instead of opinion-driven; measure and manage productivity in new ways; integrated automation enables further innovation.</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr"/>
+    </row>
+    <row r="24" ht="110" customHeight="1">
+      <c r="A24" s="18" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Southwire as customer</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>People Analytics for HR ('Igniting HR Operations at Southwire')</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Crunchr</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>https://www.crunchr.com/customers/southwire/</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>HR team faced scattered, unreliable workforce data; adopted Crunchr people-analytics platform to centralize workforce insights.</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>Platform integrated within ~1 month - significantly faster than the internal-build timeline quoted by Southwire's own BI team.</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>Faster, more consistent workforce insights; better decision-making; strong vendor support vs slower internal build.</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="inlineStr"/>
+    </row>
+    <row r="25" ht="110" customHeight="1">
+      <c r="A25" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Southwire as customer</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>B2B Demand Generation ('Establishing a Digital Baseline')</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Marsden Marketing</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>https://www.marsdenmarketing.com/case-study-establishing-a-digital-baseline</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>Digital marketing program (microsites, SEO, lead gen) for Southwire's Power Systems &amp; Solutions group across three business verticals.</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>259% increase in lead database across all three verticals; all three microsites on page 1 of Google for competitive keywords; lead-gen goals exceeded in each vertical.</t>
+        </is>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Measurable digital baseline and pipeline growth for an industrial B2B business unit.</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr"/>
+    </row>
+    <row r="26" ht="110" customHeight="1">
+      <c r="A26" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Southwire as customer</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>Facility Services</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Millennium Facility Services (MFS / MillenniumOS)</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>https://millfac.com/case-studies/southwire</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>Outsourced facility services across Southwire buildings with autonomous equipment optimization and production-aligned cleaning schedules.</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>11% under contracted budget; 35% reduction in cleaning-related production downtime; 99.7% GPS-verified task-completion rate; 100% Avetta compliance with zero audit deficiencies.</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>Lower facility cost with verifiable execution and less interference with production.</t>
+        </is>
+      </c>
+      <c r="I26" s="19" t="inlineStr"/>
+    </row>
+    <row r="27" ht="110" customHeight="1">
+      <c r="A27" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Southwire as customer</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>Recruitment Marketing - Bremen, IN Plant</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>Federated Media</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="inlineStr">
+        <is>
+          <t>https://info.federatedmedia.com/southwire-case-study</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>New 250,000 sq ft facility in Bremen, Indiana needed 100 positions filled immediately in a tight labor market; high-frequency radio ads (WRBR, WBYT, WAOR) plus on-site hiring event.</t>
+        </is>
+      </c>
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>Hiring-event turnout exceeded expectations; job offers extended to 2x as many prospective employees as initially hoped.</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>Fast, high-volume hourly recruitment for a new plant using targeted local media.</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr"/>
+    </row>
+    <row r="28" ht="110" customHeight="1">
+      <c r="A28" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Southwire as customer</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>Employee Well-Being (GRI Sustainability Case)</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>SustainCase</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>https://sustaincase.com/case-study-how-southwire-promotes-employee-well-being/</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t>Analysis of how Southwire promotes employee well-being (health, safety, wellness) based on GRI-standard sustainability reporting.</t>
+        </is>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>Qualitative; references Southwire's published sustainability metrics (southwire.com Metrics at a Glance).</t>
+        </is>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>Employer-of-choice positioning and workforce sustainability as a business asset.</t>
+        </is>
+      </c>
+      <c r="I28" s="19" t="inlineStr"/>
+    </row>
+    <row r="29" ht="110" customHeight="1">
+      <c r="A29" s="18" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>Southwire as customer</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
         <is>
           <t>Product Data Upgrade &amp; Syndication</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>IDEA (Industry Data Exchange Association)</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>https://idea4industry.com/wp-content/uploads/Southwire_case_study.pdf</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F29" s="19" t="inlineStr">
         <is>
           <t>How Southwire upgraded and syndicated its product content/data to distributors through the IDEA ecosystem.</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G29" s="19" t="inlineStr">
         <is>
           <t>See PDF (data-quality / syndication coverage improvements).</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H29" s="19" t="inlineStr">
         <is>
           <t>Clean, syndicated product data improves distributor experience and channel sales.</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13" ht="110" customHeight="1">
-      <c r="A13" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="I29" s="19" t="inlineStr"/>
+    </row>
+    <row r="30" ht="110" customHeight="1">
+      <c r="A30" s="18" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
         <is>
           <t>Southwire as customer</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C30" s="19" t="inlineStr">
         <is>
           <t>SAP Alliance Services</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>IBM</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>https://www.ibm.com/case-studies/southwire-sap-alliance-services</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F30" s="19" t="inlineStr">
         <is>
           <t>IBM services engagement supporting Southwire's SAP landscape.</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>Not surfaced in search results; see IBM case-studies page.</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H30" s="19" t="inlineStr">
         <is>
           <t>Enterprise-grade partner support for the SAP core underpinning Southwire's digital-first strategy.</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14" ht="110" customHeight="1">
-      <c r="A14" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Southwire-published (utility)</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>C7 Overhead Conductor - River Crossing</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Southwire</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>https://www.southwire.com/Utility-Whitepapers-CaseStudy</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Riverbank erosion forced a support structure move, increasing a river-crossing span from 1,290 ft to 1,840 ft; ACSR would have sagged too much, requiring larger structures and foundations, so the utility used C7 carbon-fiber composite-core conductor.</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Span increased ~43% (1,290 to 1,840 ft) with no increase in sag; avoided full line rebuild and new foundations; 40+ year service-life expectancy; single-failure-tolerant multi-stranded core.</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Higher capacity and superior sag/tension performance let utilities reuse existing structures and cut total project cost.</t>
-        </is>
-      </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>See also Utility Dive sponsored article on composite core conductors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="110" customHeight="1">
-      <c r="A15" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Southwire-published (utility)</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Novinium Cable Rejuvenation - Salt River Project</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Southwire (Novinium Underground Services)</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>https://www.southwire.com/Utility-Whitepapers-CaseStudy</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Salt River Project (utility serving south Phoenix, AZ) had aging feeder and URD cable with rising maintenance costs; chose Novinium cable rejuvenation instead of replacement.</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Less than 1% post-rejuvenation failure rate.</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Rejuvenation extends cable life at a fraction of replacement cost with minimal customer disruption.</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Salt River Project Whitepaper PDF on southwire.com.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="110" customHeight="1">
-      <c r="A16" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Southwire-published (utility)</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Novinium Modular Injection Component (MIC) - Mountain View Electric Association</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Southwire (Novinium Underground Services)</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>https://www.southwire.com/Utility-Whitepapers-CaseStudy</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>MVEA (Colorado co-op; 50,000+ members, 5,000 sq mi, ~600 miles of aging unjacketed XLPE URD cable) used the MIC - first 200A accessory enabling energized SPR injection of MV cables; developed with Richards Manufacturing.</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>Full rejuvenation of radial segments within the standard 2-hour outage window normally reserved just for testing; improved crew productivity (crews move on while injection continues).</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Energized injection means shorter outages, higher crew productivity, less rate-payer disruption than replacement or de-energized rejuvenation.</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr"/>
-    </row>
-    <row r="17" ht="110" customHeight="1">
-      <c r="A17" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Southwire-published (utility)</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Novinium Underground Services - Dayton</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Southwire (Novinium Underground Services)</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>https://www.southwire.com/Utility-Whitepapers-CaseStudy</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Additional Novinium underground cable-rejuvenation deployment (Dayton); companion to the SRP and MIC studies.</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>See PDF.</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Rejuvenate-vs-replace economics applied at another utility.</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr"/>
-    </row>
-    <row r="18" ht="110" customHeight="1">
-      <c r="A18" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Southwire-published (utility)</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Digital Grid Resiliency - Northeast US Investor-Owned Utility</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Southwire</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>https://www.southwire.com/services/digital-grid-resiliency-assessments</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Northeast US IOU worked with Southwire over several years, evaluating circuits and applying an enhanced grid-resiliency program to a subset; AI-assisted assessment mines outage and GIS data to classify outage root causes at device level.</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>Assessment identifies reliability improvements in as little as 30 days; prescriptive recommendations include cost justification and expected reliability gains.</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Data/AI-driven, device-level targeting of grid-hardening spend instead of blanket programs.</t>
-        </is>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>'Volatile to Resilient' case study PDF on the whitepapers index; Utility Dive sponsored article.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="110" customHeight="1">
-      <c r="A19" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Contractor Solutions / jobsite</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>SIMpull Solutions / Contractor Solutions Program</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>Southwire</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>https://www.southwire.com/services/contractor-solutions</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>Jobsite productivity system - SIMpull CoilPAK payoffs, SIMpull BARREL drums, SIMpull REEL, NoLube SIMpull THHN, MAXIS pulling equipment - plus Contractor Solutions Professionals (CSPs) consulting on layouts, pulling calcs, and setup for the project duration.</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>Up to 50% jobsite efficiency/savings claimed; SIMpull REEL setup ~4x faster (no jack stands, fewer people, multiple runs per reel); MAXIS: 1-man 39-min pull vs 45 min for traditional 2-man setup.</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>Beat branch-circuit wiring budgets by cutting material handling, setup time, and crew size.</t>
-        </is>
-      </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>Detailed per-project case studies appear to live with CSP team / Solutions Partner Distributors, not published openly - request internally.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="110" customHeight="1">
-      <c r="A20" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Contractor Solutions / jobsite</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>Data Center Solutions (QWIK Whips, Cabling Solutions)</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Southwire</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>https://www.southwire.com/industries/data-centers</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>Pre-assembled QWIK Whip cables and cable-pulling solutions for data center builds; positions Southwire on labor reduction and schedule for hyperscale/AI construction.</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>Publicly qualitative (streamlined ordering/install/assembly, labor cost management); no published quantified project case study found.</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>Reduce constrained field labor and keep data center projects on schedule.</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Gap the internal Advanced Conductor Value Prop deck is designed to fill.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="110" customHeight="1">
-      <c r="A21" s="13" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>Internal - Adv. Conductor Value Prop</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>C7 Corridor Upgrade - Reconductor vs Rebuild (Illustrative 25-mile Corridor)</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>Internal deck (user-shared slides, 2026-08-18)</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr"/>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>Executive value-prop model: reconductoring an existing 25-mile corridor with C7 vs traditional new-build. Existing towers and ROW reused - only the conductor changes ('same towers, same right-of-way - a stronger line, delivered in a fraction of the time').</t>
-        </is>
-      </c>
-      <c r="G21" s="14" t="inlineStr">
-        <is>
-          <t>~$57.5M capital avoided ($87.5M new-build to $30.0M C7); 6 years faster to capacity (~2 vs ~8 yrs); +450 MVA (2.5x throughput, 300 to 750 MVA). Breakdown: ~$30.0M structures/foundations, ~$15.0M ROW/permitting/legal, ~$7.5M materials efficiency, ~$5.0M labor/construction.</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="inlineStr">
-        <is>
-          <t>Faster, lower-risk capacity expansion on corridors the utility already owns - a capacity solution, not a conductor purchase.</t>
-        </is>
-      </c>
-      <c r="I21" s="14" t="inlineStr">
-        <is>
-          <t>Assumptions: baseline 300 MVA; C7 at 2.5x; structure &amp; ROW reuse; illustrative figures only. Deck defines 4 validation cases: 1) Reconductor vs Rebuild, 2) New Build, 3) Crossing, 4) Line Loss Reduction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="110" customHeight="1">
-      <c r="A22" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>Internal - Adv. Conductor Value Prop</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>Prefab Cable for Modular Cooling OEMs (Vertiv-style Archetype)</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>Internal deck (user-shared slides, 2026-08-18)</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr"/>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>Cooling is the critical path in AI &amp; hyperscale deployments; Southwire prefab electrical scope (skid-mounted, factory-tested, pre-routed power &amp; controls cable, plug-and-play CDU/chiller hookup) vs traditional field integration (field piping/brazing/welding, field-run controls, refrigerant/balancing/testing, multi-trade risk).</t>
-        </is>
-      </c>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>Onsite deployment 6-10 weeks vs 4-6+ months traditional; 2-4 months schedule compression.</t>
-        </is>
-      </c>
-      <c r="H22" s="14" t="inlineStr">
-        <is>
-          <t>Earlier customer energization, lower commissioning risk, repeatable across fleets; combined story: accelerate capacity while reducing dependence on constrained field labor.</t>
-        </is>
-      </c>
-      <c r="I22" s="14" t="inlineStr">
-        <is>
-          <t>Illustrative; Vertiv referenced as representative modular cooling OEM partner archetype.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="110" customHeight="1">
-      <c r="A23" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>Internal - Adv. Conductor Value Prop</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>Prefab Cable for Power Distribution Skid Providers</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>Internal deck (user-shared slides, 2026-08-18)</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr"/>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>Illustrative 50 MW distribution skid deployment block; loaded field labor at $180/hr. Traditional field build (15 electricians x 10 wks; weather/rework/multi-trade risk) vs Southwire prefab (pre-tested, pre-labeled harnesses; plug-and-play modular connections).</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>Install + commissioning 2-4 wks vs 8-12 wks; 40-60% fewer onsite labor hours; per block: 6-8 wks faster to energization, $500K-$800K field labor savings (vs ~$1.1M-$1.5M traditional); lower rework, faster revenue recognition, reduced LD exposure.</t>
-        </is>
-      </c>
-      <c r="H23" s="14" t="inlineStr">
-        <is>
-          <t>Faster energization and lower labor cost per repeatable deployment block. Targets: data centers, utility substations, battery storage, AI infrastructure, modular industrial plants, fuel cell &amp; gen-set OEMs.</t>
-        </is>
-      </c>
-      <c r="I23" s="14" t="inlineStr">
-        <is>
-          <t>Figures directional - validate with partner labor data.</t>
-        </is>
-      </c>
+      <c r="I30" s="19" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:I23"/>
+  <autoFilter ref="A3:I30"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -1488,9 +1831,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1502,7 +1852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1510,100 +1860,124 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Southwire Case Studies - Read Me</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr"/>
+      <c r="B1" s="22" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr"/>
-      <c r="B2" s="16" t="inlineStr"/>
+      <c r="A2" s="22" t="inlineStr"/>
+      <c r="B2" s="22" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Southwire-published (utility)</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Case study published by Southwire about its own utility products/services delivering customer outcomes - most relevant to the Advanced Conductor Value Prop objective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Southwire-published (services)</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Southwire SPEED / CableTechSupport service case studies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>Contractor Solutions / jobsite</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Southwire jobsite-productivity case studies (SIMpull, data centers). Named case-study PDFs live on the Contractor Solutions page; more are held by the CSP team / distributors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Southwire-published (corporate)</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Corporate/shared-value case studies (e.g. Harvard 12 for Life).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Internal - Adv. Conductor Value Prop</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>From the internal 'Advanced Conductor Value Prop Project' deck (slides shared 2026-08-18). Illustrative figures only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Southwire as customer</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Case study published by a vendor/partner featuring Southwire as the customer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Southwire-published (utility)</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Case study published by Southwire about its own utility products/services.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Contractor Solutions / jobsite</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Southwire jobsite-productivity material (SIMpull, data centers). Detailed project case studies are held by the CSP team / distributors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Internal - Adv. Conductor Value Prop</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>From the internal 'Advanced Conductor Value Prop Project' deck (slides shared 2026-08-18). Illustrative figures only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr"/>
-      <c r="B8" s="16" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Case study published by a vendor/partner featuring Southwire as the customer (background only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr"/>
+      <c r="B10" s="22" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>Rockwell, SAP, IBM, Marsden, MFS and southwire.com pages could not be fetched directly (network restrictions); their entries are built from search-engine content of those pages. Rows marked 'See PDF/page' have additional numbers in the linked document.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>Companion file</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>SOUTHWIRE_CASE_STUDIES.md in the shardt87/ln repo, branch claude/southwire-case-studies-x8sv7p.</t>
         </is>

</xml_diff>